<commit_message>
feat: Enhance bulk grade upload by improving metadata extraction and adding conditional formatting for grades
</commit_message>
<xml_diff>
--- a/grading/templates/grades_upload_marking_periods.xlsx
+++ b/grading/templates/grades_upload_marking_periods.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dewardseneh/workdir/dewx/webapps/highschool/backend-2/grading/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B4D568E-6B27-1C49-9292-95515974570B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202D3B54-1BA1-D140-B274-BFDF4D984B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Grades Upload" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Grades Upload'!$A$1:$M$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Grades Upload'!$A$1:$M$41</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="19">
   <si>
     <t>Grade Level:</t>
   </si>
@@ -77,6 +77,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Subject Name:</t>
   </si>
 </sst>
 </file>
@@ -581,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
@@ -642,7 +645,7 @@
     </row>
     <row r="4" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -658,7 +661,9 @@
       <c r="M4" s="2"/>
     </row>
     <row r="5" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
+      <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -672,82 +677,60 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="1:13" ht="40" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+    </row>
+    <row r="7" spans="1:13" ht="40" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="L6" s="9" t="s">
+      <c r="L7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="9" t="s">
+      <c r="M7" s="9" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="K7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="L7" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="M7" s="13" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.2">
@@ -765,7 +748,7 @@
       <c r="F8" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="12" t="s">
         <v>17</v>
       </c>
       <c r="H8" s="11" t="s">
@@ -901,7 +884,9 @@
     <row r="12" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
-      <c r="C12" s="11"/>
+      <c r="C12" s="11" t="s">
+        <v>17</v>
+      </c>
       <c r="D12" s="11" t="s">
         <v>17</v>
       </c>
@@ -936,9 +921,7 @@
     <row r="13" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
-      <c r="C13" s="11" t="s">
-        <v>17</v>
-      </c>
+      <c r="C13" s="11"/>
       <c r="D13" s="11" t="s">
         <v>17</v>
       </c>
@@ -1969,11 +1952,48 @@
         <v>17</v>
       </c>
     </row>
+    <row r="41" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="10"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G41" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="J41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K41" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="L41" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="M41" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0" right="1.38888888888889E-2" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="75" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
-    <ignoredError sqref="A1 A4 A3 C3:M3 C7:M11 C13:M40 D12:M12 A6 C6:M6 C4:M4 A2 C2:M2 C1:M1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1 A5 A3 C3:M3 C8:M12 C14:M41 D13:M13 A7 C7:M7 C5:M5 A2 C2:M2 C1:M1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>